<commit_message>
Price offered testcases modification
</commit_message>
<xml_diff>
--- a/uploads/Bid_file_success_error_newly_updated (12).xlsx
+++ b/uploads/Bid_file_success_error_newly_updated (12).xlsx
@@ -540,7 +540,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="str">
-        <v>TestSigma_13-03-2026_SC1_H1_854</v>
+        <v>TestSigma_16-03-2026_SC1_G6_224</v>
       </c>
       <c r="B2" s="1">
         <v>2001</v>
@@ -654,7 +654,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="str">
-        <v>TestSigma_13-03-2026_SC1_XQ_446</v>
+        <v>TestSigma_16-03-2026_SC1_0H_862</v>
       </c>
       <c r="B3" s="1">
         <v>2001</v>
@@ -768,7 +768,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="str">
-        <v>TestSigma_13-03-2026_SC1_44_189</v>
+        <v>TestSigma_16-03-2026_SC1_HH_639</v>
       </c>
       <c r="B4" s="1">
         <v>2001</v>
@@ -881,7 +881,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="str">
-        <v>TestSigma_13-03-2026_SC1_OB_856</v>
+        <v>TestSigma_16-03-2026_SC1_9N_416</v>
       </c>
       <c r="B5" s="1">
         <v>2001</v>
@@ -994,7 +994,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="str">
-        <v>TestSigma_13-03-2026_SC1_5Z_603</v>
+        <v>TestSigma_16-03-2026_SC1_B4_168</v>
       </c>
       <c r="B6" s="1">
         <v>2001</v>

</xml_diff>

<commit_message>
commitment list testcases modification
</commit_message>
<xml_diff>
--- a/uploads/Bid_file_success_error_newly_updated (12).xlsx
+++ b/uploads/Bid_file_success_error_newly_updated (12).xlsx
@@ -540,7 +540,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="str">
-        <v>TestSigma_16-03-2026_SC1_G6_224</v>
+        <v>TestSigma_17-03-2026_SC1_BR_687</v>
       </c>
       <c r="B2" s="1">
         <v>2001</v>
@@ -654,7 +654,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="str">
-        <v>TestSigma_16-03-2026_SC1_0H_862</v>
+        <v>TestSigma_17-03-2026_SC1_AI_621</v>
       </c>
       <c r="B3" s="1">
         <v>2001</v>
@@ -768,7 +768,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="str">
-        <v>TestSigma_16-03-2026_SC1_HH_639</v>
+        <v>TestSigma_17-03-2026_SC1_9N_774</v>
       </c>
       <c r="B4" s="1">
         <v>2001</v>
@@ -881,7 +881,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="str">
-        <v>TestSigma_16-03-2026_SC1_9N_416</v>
+        <v>TestSigma_17-03-2026_SC1_KN_798</v>
       </c>
       <c r="B5" s="1">
         <v>2001</v>
@@ -994,7 +994,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="str">
-        <v>TestSigma_16-03-2026_SC1_B4_168</v>
+        <v>TestSigma_17-03-2026_SC1_SB_116</v>
       </c>
       <c r="B6" s="1">
         <v>2001</v>

</xml_diff>

<commit_message>
loggers and constants implementation
</commit_message>
<xml_diff>
--- a/uploads/Bid_file_success_error_newly_updated (12).xlsx
+++ b/uploads/Bid_file_success_error_newly_updated (12).xlsx
@@ -540,7 +540,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="str">
-        <v>TestSigma_17-03-2026_SC1_BR_687</v>
+        <v>TestSigma_21-03-2026_SC1_D1_526</v>
       </c>
       <c r="B2" s="1">
         <v>2001</v>
@@ -654,7 +654,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="str">
-        <v>TestSigma_17-03-2026_SC1_AI_621</v>
+        <v>TestSigma_21-03-2026_SC1_CP_922</v>
       </c>
       <c r="B3" s="1">
         <v>2001</v>
@@ -768,7 +768,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="str">
-        <v>TestSigma_17-03-2026_SC1_9N_774</v>
+        <v>TestSigma_21-03-2026_SC1_YX_863</v>
       </c>
       <c r="B4" s="1">
         <v>2001</v>
@@ -881,7 +881,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="str">
-        <v>TestSigma_17-03-2026_SC1_KN_798</v>
+        <v>TestSigma_21-03-2026_SC1_B9_716</v>
       </c>
       <c r="B5" s="1">
         <v>2001</v>
@@ -994,7 +994,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="str">
-        <v>TestSigma_17-03-2026_SC1_SB_116</v>
+        <v>TestSigma_21-03-2026_SC1_F9_719</v>
       </c>
       <c r="B6" s="1">
         <v>2001</v>

</xml_diff>

<commit_message>
Demo testplan for price offered
</commit_message>
<xml_diff>
--- a/uploads/Bid_file_success_error_newly_updated (12).xlsx
+++ b/uploads/Bid_file_success_error_newly_updated (12).xlsx
@@ -540,7 +540,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="str">
-        <v>TestSigma_26-03-2026_SC1_V7_505</v>
+        <v>TestSigma_31-03-2026_SC1_RJ_157</v>
       </c>
       <c r="B2" s="1">
         <v>2001</v>
@@ -654,7 +654,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="str">
-        <v>TestSigma_26-03-2026_SC1_99_682</v>
+        <v>TestSigma_31-03-2026_SC1_RM_600</v>
       </c>
       <c r="B3" s="1">
         <v>2001</v>
@@ -768,7 +768,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="str">
-        <v>TestSigma_26-03-2026_SC1_CX_452</v>
+        <v>TestSigma_31-03-2026_SC1_XD_895</v>
       </c>
       <c r="B4" s="1">
         <v>2001</v>
@@ -881,7 +881,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="str">
-        <v>TestSigma_26-03-2026_SC1_12_918</v>
+        <v>TestSigma_31-03-2026_SC1_I5_795</v>
       </c>
       <c r="B5" s="1">
         <v>2001</v>
@@ -994,7 +994,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="str">
-        <v>TestSigma_26-03-2026_SC1_GZ_590</v>
+        <v>TestSigma_31-03-2026_SC1_MC_930</v>
       </c>
       <c r="B6" s="1">
         <v>2001</v>

</xml_diff>

<commit_message>
pre-requites and testplan commitment list
</commit_message>
<xml_diff>
--- a/uploads/Bid_file_success_error_newly_updated (12).xlsx
+++ b/uploads/Bid_file_success_error_newly_updated (12).xlsx
@@ -540,7 +540,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="str">
-        <v>TestSigma_31-03-2026_SC1_RJ_157</v>
+        <v>TestSigma_01-04-2026_SC1_JI_899</v>
       </c>
       <c r="B2" s="1">
         <v>2001</v>
@@ -654,7 +654,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="str">
-        <v>TestSigma_31-03-2026_SC1_RM_600</v>
+        <v>TestSigma_01-04-2026_SC1_L4_750</v>
       </c>
       <c r="B3" s="1">
         <v>2001</v>
@@ -768,7 +768,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="str">
-        <v>TestSigma_31-03-2026_SC1_XD_895</v>
+        <v>TestSigma_01-04-2026_SC1_29_597</v>
       </c>
       <c r="B4" s="1">
         <v>2001</v>
@@ -881,7 +881,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="str">
-        <v>TestSigma_31-03-2026_SC1_I5_795</v>
+        <v>TestSigma_01-04-2026_SC1_7M_239</v>
       </c>
       <c r="B5" s="1">
         <v>2001</v>
@@ -994,7 +994,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="str">
-        <v>TestSigma_31-03-2026_SC1_MC_930</v>
+        <v>TestSigma_01-04-2026_SC1_D9_383</v>
       </c>
       <c r="B6" s="1">
         <v>2001</v>

</xml_diff>

<commit_message>
price offered testcases modification-7done
</commit_message>
<xml_diff>
--- a/uploads/Bid_file_success_error_newly_updated (12).xlsx
+++ b/uploads/Bid_file_success_error_newly_updated (12).xlsx
@@ -540,7 +540,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="str">
-        <v>TestSigma_01-04-2026_SC1_JI_899</v>
+        <v>TestSigma_02-04-2026_SC1_1K_869</v>
       </c>
       <c r="B2" s="1">
         <v>2001</v>
@@ -654,7 +654,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="str">
-        <v>TestSigma_01-04-2026_SC1_L4_750</v>
+        <v>TestSigma_02-04-2026_SC1_KJ_344</v>
       </c>
       <c r="B3" s="1">
         <v>2001</v>
@@ -768,7 +768,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="str">
-        <v>TestSigma_01-04-2026_SC1_29_597</v>
+        <v>TestSigma_02-04-2026_SC1_A1_625</v>
       </c>
       <c r="B4" s="1">
         <v>2001</v>
@@ -881,7 +881,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="str">
-        <v>TestSigma_01-04-2026_SC1_7M_239</v>
+        <v>TestSigma_02-04-2026_SC1_QJ_363</v>
       </c>
       <c r="B5" s="1">
         <v>2001</v>
@@ -994,7 +994,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="str">
-        <v>TestSigma_01-04-2026_SC1_D9_383</v>
+        <v>TestSigma_02-04-2026_SC1_8L_619</v>
       </c>
       <c r="B6" s="1">
         <v>2001</v>

</xml_diff>

<commit_message>
testplan modification and testcases
</commit_message>
<xml_diff>
--- a/uploads/Bid_file_success_error_newly_updated (12).xlsx
+++ b/uploads/Bid_file_success_error_newly_updated (12).xlsx
@@ -540,7 +540,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="str">
-        <v>TestSigma_02-04-2026_SC1_1K_869</v>
+        <v>TestSigma_06-04-2026_SC1_AN_982</v>
       </c>
       <c r="B2" s="1">
         <v>2001</v>
@@ -654,7 +654,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="str">
-        <v>TestSigma_02-04-2026_SC1_KJ_344</v>
+        <v>TestSigma_06-04-2026_SC1_U5_897</v>
       </c>
       <c r="B3" s="1">
         <v>2001</v>
@@ -768,7 +768,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="str">
-        <v>TestSigma_02-04-2026_SC1_A1_625</v>
+        <v>TestSigma_06-04-2026_SC1_XH_941</v>
       </c>
       <c r="B4" s="1">
         <v>2001</v>
@@ -881,7 +881,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="str">
-        <v>TestSigma_02-04-2026_SC1_QJ_363</v>
+        <v>TestSigma_06-04-2026_SC1_JK_346</v>
       </c>
       <c r="B5" s="1">
         <v>2001</v>
@@ -994,7 +994,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="str">
-        <v>TestSigma_02-04-2026_SC1_8L_619</v>
+        <v>TestSigma_06-04-2026_SC1_3F_588</v>
       </c>
       <c r="B6" s="1">
         <v>2001</v>

</xml_diff>

<commit_message>
general settings and bid map testcases modification
</commit_message>
<xml_diff>
--- a/uploads/Bid_file_success_error_newly_updated (12).xlsx
+++ b/uploads/Bid_file_success_error_newly_updated (12).xlsx
@@ -540,7 +540,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="str">
-        <v>TestSigma_06-04-2026_SC1_AN_982</v>
+        <v>TestSigma_29-04-2026_SC1_5Q_823</v>
       </c>
       <c r="B2" s="1">
         <v>2001</v>
@@ -654,7 +654,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="str">
-        <v>TestSigma_06-04-2026_SC1_U5_897</v>
+        <v>TestSigma_29-04-2026_SC1_UW_671</v>
       </c>
       <c r="B3" s="1">
         <v>2001</v>
@@ -768,7 +768,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="str">
-        <v>TestSigma_06-04-2026_SC1_XH_941</v>
+        <v>TestSigma_29-04-2026_SC1_V6_237</v>
       </c>
       <c r="B4" s="1">
         <v>2001</v>
@@ -881,7 +881,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="str">
-        <v>TestSigma_06-04-2026_SC1_JK_346</v>
+        <v>TestSigma_29-04-2026_SC1_J9_355</v>
       </c>
       <c r="B5" s="1">
         <v>2001</v>
@@ -994,7 +994,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="str">
-        <v>TestSigma_06-04-2026_SC1_3F_588</v>
+        <v>TestSigma_29-04-2026_SC1_Z7_946</v>
       </c>
       <c r="B6" s="1">
         <v>2001</v>

</xml_diff>